<commit_message>
Add Phase 5a: visual page preview, formatting toolbar, outline panel
CSS-based page-height seam approximation (no real reflow -- confirmed
scope with Boril), a Tiptap-backed rich-text toolbar (bold/italic/font/
size/alignment/lists/undo-redo, local to the browser), and a clickable
heading outline. Also fixes a pre-existing lint error in the documents
page (JSX constructed inside try/catch).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-tracker.xlsx
+++ b/roadmap-tracker.xlsx
@@ -1131,10 +1131,14 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>CSS visual approximation (repeating-linear-gradient shadow seam every page-height, computed from pageSize/orientation) in one continuous scroll container -- NOT real reflow; confirmed with Boril before starting Phase 5 that true live-reflowing pagination on Tiptap/ProseMirror is a separate, much larger project</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -1145,10 +1149,14 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>components/Toolbar.tsx -- bold/italic/underline/strike/font-family/font-size/alignment/lists/undo-redo via direct Tiptap commands; local-only, not routed through backend FormattingRule system (that's Phase 5b's Properties-panel job)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
@@ -1173,10 +1181,14 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>components/OutlinePanel.tsx -- lists headings by level, click scrolls via data-element-id (new editor/elementId.ts extension); hidden below lg breakpoint on small screens</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
@@ -1192,7 +1204,7 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Tiptap-ов базов text undo/redo вече работи (Ctrl+Z); истинската history/versioning система още не</t>
+          <t>Tiptap-ов базов text undo/redo вече работи и вече е и кликаема toolbar бутони (не само Ctrl+Z); истинската history/versioning система за formatting/structural промени още не (Phase 5b)</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1602,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Текстово редактиране работи (Tiptap); индиректно oформление през template/инструкции вече работи; директен per-element Properties panel остава Phase 5</t>
+          <t>Toolbar (bold/italic/underline/strike/font/size/alignment/lists) + template/instructions от Phase 4 -- всичко все още само локално в браузъра, няма save endpoint</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Phase 5: live overrides, formatting undo/redo, conflict modal
Properties panel for per-element style overrides (spec 7.9 tier 1,
persisted server-side, wins over templates/instructions, survives a
reformat), a separate backend undo/redo history for formatting and
structural changes, and the full Conflict Resolution modal (spec
7.10) with per-conflict Apply-recommended/Keep-current choices.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-tracker.xlsx
+++ b/roadmap-tracker.xlsx
@@ -1167,10 +1167,14 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>components/PropertiesPanel.tsx -- edits the selected element's style directly (spec §7.9 tier 1), persisted via PATCH/DELETE .../elements/{id}/style; wins over template/instructions automatically (NFR-008), survives a reformat</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -1199,12 +1203,12 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Tiptap-ов базов text undo/redo вече работи и вече е и кликаема toolbar бутони (не само Ctrl+Z); истинската history/versioning система за formatting/structural промени още не (Phase 5b)</t>
+          <t>Tiptap text undo/redo (Ctrl+Z, toolbar buttons) плюс отделен formatting/structural undo/redo stack (DocumentService, full Document snapshots) за /format и elements/{id}/style -- двете истории са напълно независими една от друга</t>
         </is>
       </c>
     </row>
@@ -1217,10 +1221,14 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>components/ConflictModal.tsx -- пълна версия по §7.10 (Required/Current + Apply recommended/Keep current поотделно за всеки конфликт); detect_conflicts() в backend, /format връща 409 вместо тихо прилагане, ако има неразрешени конфликти</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1286,7 +1294,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>78 pytest теста към момента (Phase 0-1-2-3-4); ще растат с всяка следваща фаза</t>
+          <t>96 pytest теста към момента (Phase 0-1-2-3-4-5); Phase 5 е изцяло завършена</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1615,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Toolbar (bold/italic/underline/strike/font/size/alignment/lists) + template/instructions от Phase 4 -- всичко все още само локално в браузъра, няма save endpoint</t>
+          <t>Текстово редактиране (Tiptap) + Toolbar (локално) + Properties panel с live per-element override (персистирано, печели над template/instructions по priority)</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1627,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Само Tiptap-овия базов text undo/redo (Ctrl+Z)</t>
+          <t>Tiptap текстов undo/redo (Ctrl+Z + toolbar) + отделен formatting/structural undo/redo (backend snapshot stack, /undo и /redo endpoints)</t>
         </is>
       </c>
     </row>
@@ -1636,12 +1644,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Приоритетите се решават детерминистично и тихо (по-нисък priority номер печели) -- самата Conflict modal остава Phase 5</t>
+          <t>ConflictModal.tsx -- пълна версия по §7.10, Required/Current + Apply recommended/Keep current поотделно за всеки конфликт; /format връща 409 вместо тихо избиране</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Phase 6: DOCX and PDF export
Two independent exporters reading the same document.resolvedStyles
the editor already renders: docx_export.py (python-docx) produces a
real editable Word document with heading/paragraph/list/table/image/
code-block content and page setup; pdf_export.py (reportlab, new
dependency) produces a real PDF via its flowable model, with header/
footer/page-number canvas callbacks. LibreOffice is unavailable on
this machine, so this is two independent renderers rather than a
DOCX-to-PDF conversion pipeline -- a flagged, documented tradeoff
(PDF fonts are substituted, not embedded).

GET /api/documents/{id}/export/docx and .../export/pdf return the
file directly with a download Content-Disposition header; ExportPanel.tsx
adds two plain download links next to the formatting panel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-tracker.xlsx
+++ b/roadmap-tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Acceptance Criteria" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Criteria" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1243,10 +1243,14 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>backend/app/export/docx_export.py -- python-docx, чете същите resolvedStyles, които editor-ът вече рендва; headings/paragraphs/lists/tables/images/code blocks + page setup (size/margини/orientation/header-footer/page numbers, последното чрез raw-XML PAGE field). Известно опростяване: list nesting отвъд Word-овите вградени List Bullet/List Number стилове е приближено чрез left_indent, не истинско multi-level numbering.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -1257,10 +1261,14 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>backend/app/export/pdf_export.py -- reportlab (нова pip зависимост, чист Python, без системен install). LibreOffice/soffice не е наличен на тази машина (проверено директно) и docx/xlsx skill-овете's soffice.py wrapper е Linux-only -- затова PDF е напълно отделен exporter, не DOCX-to-PDF конверсия. Известна граница: reportlab няма вградени TrueType шрифтове отвъд Helvetica/Times/Courier, така че PDF шрифтовете са substituted, не пиксел-идентични с preview/DOCX.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n"/>
@@ -1271,10 +1279,14 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>backend/tests/test_docx_export.py + test_pdf_export.py -- round-trip четене (python-docx / pypdf) на build_docx()/build_pdf() резултат; GET .../export/docx и .../export/pdf тествани в test_documents_api.py (200 + правилен Content-Type/Content-Disposition, 404 за непознат документ). Живо потвърдено в браузъра: template + heading/list/table документ -&gt; сваляне на двата файла -&gt; DOCX прочетен обратно (heading style/bold+italic runs/list style/table cells/margини съвпадат с academic-default), PDF отворен през pypdf text-extraction (1 страница, целият текст присъства в правилния ред).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1294,7 +1306,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>96 pytest теста към момента (Phase 0-1-2-3-4-5); Phase 5 е изцяло завършена</t>
+          <t>104 pytest теста към момента (Phase 0-1-2-3-4-5-6); Phase 6 е изцяло завършена</t>
         </is>
       </c>
     </row>
@@ -1661,10 +1673,14 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>GET /api/documents/{id}/export/docx -- build_docx() (python-docx) връща реален, редактируем .docx с heading/paragraph/list/table/image/code-block съдържание и page setup; потвърдено чрез round-trip тест + живо сваляне и повторно четене</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1674,10 +1690,14 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>GET /api/documents/{id}/export/pdf -- build_pdf() (reportlab) връща валиден PDF; шрифтовете са substituted (Helvetica/Times/Courier), не ембеднати истински .ttf файлове -- флагнато като известна граница, не бъг</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">

</xml_diff>